<commit_message>
fix scorecard scale & StandardScoreTransformer
</commit_message>
<xml_diff>
--- a/examples/model_report/credit_scorecard_report.xlsx
+++ b/examples/model_report/credit_scorecard_report.xlsx
@@ -6497,7 +6497,7 @@
       <c r="C68" s="9" t="inlineStr"/>
       <c r="D68" s="9" t="inlineStr">
         <is>
-          <t>repairs,furniture/equipment</t>
+          <t>furniture/equipment,repairs</t>
         </is>
       </c>
       <c r="E68" s="9" t="n">
@@ -6625,7 +6625,7 @@
       <c r="C70" s="9" t="inlineStr"/>
       <c r="D70" s="9" t="inlineStr">
         <is>
-          <t>others,education,car (new),domestic appliances</t>
+          <t>domestic appliances,education,others,car (new)</t>
         </is>
       </c>
       <c r="E70" s="9" t="n">
@@ -7069,7 +7069,7 @@
       <c r="C79" s="9" t="inlineStr"/>
       <c r="D79" s="9" t="inlineStr">
         <is>
-          <t>retraining,others,business,domestic appliances</t>
+          <t>retraining,domestic appliances,business,others</t>
         </is>
       </c>
       <c r="E79" s="9" t="n">
@@ -7197,7 +7197,7 @@
       <c r="C81" s="9" t="inlineStr"/>
       <c r="D81" s="9" t="inlineStr">
         <is>
-          <t>repairs,furniture/equipment</t>
+          <t>furniture/equipment,repairs</t>
         </is>
       </c>
       <c r="E81" s="9" t="n">
@@ -11765,7 +11765,7 @@
       <c r="C254" s="7" t="inlineStr"/>
       <c r="D254" s="7" t="inlineStr">
         <is>
-          <t>delay in paying off in the past,critical account/ other credits existing (not at this bank)</t>
+          <t>critical account/ other credits existing (not at this bank),delay in paying off in the past</t>
         </is>
       </c>
       <c r="E254" s="7" t="n">
@@ -11829,7 +11829,7 @@
       <c r="C255" s="9" t="inlineStr"/>
       <c r="D255" s="9" t="inlineStr">
         <is>
-          <t>no credits taken/ all credits paid back duly,existing credits paid back duly till now,all credits at this bank paid back duly</t>
+          <t>no credits taken/ all credits paid back duly,all credits at this bank paid back duly,existing credits paid back duly till now</t>
         </is>
       </c>
       <c r="E255" s="9" t="n">
@@ -12213,7 +12213,7 @@
       <c r="C263" s="7" t="inlineStr"/>
       <c r="D263" s="7" t="inlineStr">
         <is>
-          <t>delay in paying off in the past,no credits taken/ all credits paid back duly,all credits at this bank paid back duly</t>
+          <t>delay in paying off in the past,all credits at this bank paid back duly,no credits taken/ all credits paid back duly</t>
         </is>
       </c>
       <c r="E263" s="7" t="n">
@@ -16437,7 +16437,7 @@
     <row r="10">
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>{'base_odds': 35, 'base_score': 750, 'combiner': &lt;toad.transform.Combiner object at 0x0000023A49D0B560&gt;, 'pdo': 60, 'pipeline__memory': None, 'pipeline__steps': [('preprocessing_select', FeatureSelection(target='creditability')), ('combiner', Combiner(min_bin_size=0.2, target='creditability')), ('transform', WOETransformer(exclude=[], target='creditability')), ('processing_select', FeatureSelection(engine='toad', target='creditability')), ('stepwise', StepwiseSelection(target='creditability')), ('logistic', ITLubberLogisticRegression(target='creditability'))], 'pipeline__transform_input': None, 'pipeline__verbose': False, 'pipeline__preprocessing_select': FeatureSelection(target='creditability'), 'pipeline__combiner': Combiner(min_bin_size=0.2, target='creditability'), 'pipeline__transform': WOETransformer(exclude=[], target='creditability'), 'pipeline__processing_select': FeatureSelection(engine='toad', target='creditability'), 'pipeline__stepwise': StepwiseSelection(target='creditability'), 'pipeline__logistic': ITLubberLogisticRegression(target='creditability'), 'pipeline__preprocessing_select__corr': 0.7, 'pipeline__preprocessing_select__empty': 0.95, 'pipeline__preprocessing_select__engine': 'scorecardpy', 'pipeline__preprocessing_select__exclude': None, 'pipeline__preprocessing_select__identical': 0.95, 'pipeline__preprocessing_select__iv': 0.02, 'pipeline__preprocessing_select__remove': None, 'pipeline__preprocessing_select__return_drop': True, 'pipeline__preprocessing_select__target': 'creditability', 'pipeline__preprocessing_select__target_rm': False, 'pipeline__combiner__adj_rules': {}, 'pipeline__combiner__empty_separate': True, 'pipeline__combiner__gamma': 0.01, 'pipeline__combiner__max_bin_size': None, 'pipeline__combiner__max_n_bins': None, 'pipeline__combiner__max_n_prebins': 20, 'pipeline__combiner__method': 'chi', 'pipeline__combiner__min_bin_size': 0.2, 'pipeline__combiner__min_n_bins': 2, 'pipeline__combiner__min_prebin_size': 0.02, 'pipeline__combiner__monotonic_trend': 'auto_asc_desc', 'pipeline__combiner__n_jobs': 1, 'pipeline__combiner__target': 'creditability', 'pipeline__transform__exclude': [], 'pipeline__transform__target': 'creditability', 'pipeline__processing_select__corr': 0.7, 'pipeline__processing_select__empty': 0.95, 'pipeline__processing_select__engine': 'toad', 'pipeline__processing_select__exclude': None, 'pipeline__processing_select__identical': 0.95, 'pipeline__processing_select__iv': 0.02, 'pipeline__processing_select__remove': None, 'pipeline__processing_select__return_drop': True, 'pipeline__processing_select__target': 'creditability', 'pipeline__processing_select__target_rm': False, 'pipeline__stepwise__criterion': 'aic', 'pipeline__stepwise__direction': 'both', 'pipeline__stepwise__estimator': 'ols', 'pipeline__stepwise__exclude': None, 'pipeline__stepwise__intercept': True, 'pipeline__stepwise__max_iter': None, 'pipeline__stepwise__p_enter': 0.01, 'pipeline__stepwise__p_remove': 0.01, 'pipeline__stepwise__p_value_enter': 0.2, 'pipeline__stepwise__return_drop': True, 'pipeline__stepwise__target': 'creditability', 'pipeline__stepwise__target_rm': False, 'pipeline__logistic__C': 1.0, 'pipeline__logistic__calculate_stats': True, 'pipeline__logistic__class_weight': None, 'pipeline__logistic__dual': False, 'pipeline__logistic__fit_intercept': True, 'pipeline__logistic__intercept_scaling': 1, 'pipeline__logistic__l1_ratio': None, 'pipeline__logistic__max_iter': 100, 'pipeline__logistic__multi_class': 'auto', 'pipeline__logistic__n_jobs': None, 'pipeline__logistic__penalty': 'l2', 'pipeline__logistic__random_state': None, 'pipeline__logistic__solver': 'lbfgs', 'pipeline__logistic__target': 'creditability', 'pipeline__logistic__tol': 0.0001, 'pipeline__logistic__verbose': 0, 'pipeline__logistic__warm_start': False, 'pipeline': Pipeline(steps=[('preprocessing_select',
+          <t>{'base_odds': 35, 'base_score': 750, 'combiner': &lt;toad.transform.Combiner object at 0x000002C34CD49310&gt;, 'pdo': 60, 'pipeline__memory': None, 'pipeline__steps': [('preprocessing_select', FeatureSelection(target='creditability')), ('combiner', Combiner(min_bin_size=0.2, target='creditability')), ('transform', WOETransformer(exclude=[], target='creditability')), ('processing_select', FeatureSelection(engine='toad', target='creditability')), ('stepwise', StepwiseSelection(target='creditability')), ('logistic', ITLubberLogisticRegression(target='creditability'))], 'pipeline__transform_input': None, 'pipeline__verbose': False, 'pipeline__preprocessing_select': FeatureSelection(target='creditability'), 'pipeline__combiner': Combiner(min_bin_size=0.2, target='creditability'), 'pipeline__transform': WOETransformer(exclude=[], target='creditability'), 'pipeline__processing_select': FeatureSelection(engine='toad', target='creditability'), 'pipeline__stepwise': StepwiseSelection(target='creditability'), 'pipeline__logistic': ITLubberLogisticRegression(target='creditability'), 'pipeline__preprocessing_select__corr': 0.7, 'pipeline__preprocessing_select__empty': 0.95, 'pipeline__preprocessing_select__engine': 'scorecardpy', 'pipeline__preprocessing_select__exclude': None, 'pipeline__preprocessing_select__identical': 0.95, 'pipeline__preprocessing_select__iv': 0.02, 'pipeline__preprocessing_select__remove': None, 'pipeline__preprocessing_select__return_drop': True, 'pipeline__preprocessing_select__target': 'creditability', 'pipeline__preprocessing_select__target_rm': False, 'pipeline__combiner__adj_rules': {}, 'pipeline__combiner__empty_separate': True, 'pipeline__combiner__gamma': 0.01, 'pipeline__combiner__max_bin_size': None, 'pipeline__combiner__max_n_bins': None, 'pipeline__combiner__max_n_prebins': 20, 'pipeline__combiner__method': 'chi', 'pipeline__combiner__min_bin_size': 0.2, 'pipeline__combiner__min_n_bins': 2, 'pipeline__combiner__min_prebin_size': 0.02, 'pipeline__combiner__monotonic_trend': 'auto_asc_desc', 'pipeline__combiner__n_jobs': 1, 'pipeline__combiner__target': 'creditability', 'pipeline__transform__exclude': [], 'pipeline__transform__target': 'creditability', 'pipeline__processing_select__corr': 0.7, 'pipeline__processing_select__empty': 0.95, 'pipeline__processing_select__engine': 'toad', 'pipeline__processing_select__exclude': None, 'pipeline__processing_select__identical': 0.95, 'pipeline__processing_select__iv': 0.02, 'pipeline__processing_select__remove': None, 'pipeline__processing_select__return_drop': True, 'pipeline__processing_select__target': 'creditability', 'pipeline__processing_select__target_rm': False, 'pipeline__stepwise__criterion': 'aic', 'pipeline__stepwise__direction': 'both', 'pipeline__stepwise__estimator': 'ols', 'pipeline__stepwise__exclude': None, 'pipeline__stepwise__intercept': True, 'pipeline__stepwise__max_iter': None, 'pipeline__stepwise__p_enter': 0.01, 'pipeline__stepwise__p_remove': 0.01, 'pipeline__stepwise__p_value_enter': 0.2, 'pipeline__stepwise__return_drop': True, 'pipeline__stepwise__target': 'creditability', 'pipeline__stepwise__target_rm': False, 'pipeline__logistic__C': 1.0, 'pipeline__logistic__calculate_stats': True, 'pipeline__logistic__class_weight': None, 'pipeline__logistic__dual': False, 'pipeline__logistic__fit_intercept': True, 'pipeline__logistic__intercept_scaling': 1, 'pipeline__logistic__l1_ratio': None, 'pipeline__logistic__max_iter': 100, 'pipeline__logistic__multi_class': 'auto', 'pipeline__logistic__n_jobs': None, 'pipeline__logistic__penalty': 'l2', 'pipeline__logistic__random_state': None, 'pipeline__logistic__solver': 'lbfgs', 'pipeline__logistic__target': 'creditability', 'pipeline__logistic__tol': 0.0001, 'pipeline__logistic__verbose': 0, 'pipeline__logistic__warm_start': False, 'pipeline': Pipeline(steps=[('preprocessing_select',
                  FeatureSelection(target='creditability')),
                 ('combiner',
                  Combiner(min_bin_size=0.2, target='creditability')),
@@ -16447,7 +16447,7 @@
                  FeatureSelection(engine='toad', target='creditability')),
                 ('stepwise', StepwiseSelection(target='creditability')),
                 ('logistic',
-                 ITLubberLogisticRegression(target='creditability'))]), 'pretrain_lr__C': 1.0, 'pretrain_lr__calculate_stats': True, 'pretrain_lr__class_weight': None, 'pretrain_lr__dual': False, 'pretrain_lr__fit_intercept': True, 'pretrain_lr__intercept_scaling': 1, 'pretrain_lr__l1_ratio': None, 'pretrain_lr__max_iter': 100, 'pretrain_lr__multi_class': 'auto', 'pretrain_lr__n_jobs': None, 'pretrain_lr__penalty': 'l2', 'pretrain_lr__random_state': None, 'pretrain_lr__solver': 'lbfgs', 'pretrain_lr__target': 'creditability', 'pretrain_lr__tol': 0.0001, 'pretrain_lr__verbose': 0, 'pretrain_lr__warm_start': False, 'pretrain_lr': ITLubberLogisticRegression(target='creditability'), 'rate': 2, 'target': 'creditability', 'transer': &lt;toad.transform.WOETransformer object at 0x0000023A496C8740&gt;}</t>
+                 ITLubberLogisticRegression(target='creditability'))]), 'pretrain_lr__C': 1.0, 'pretrain_lr__calculate_stats': True, 'pretrain_lr__class_weight': None, 'pretrain_lr__dual': False, 'pretrain_lr__fit_intercept': True, 'pretrain_lr__intercept_scaling': 1, 'pretrain_lr__l1_ratio': None, 'pretrain_lr__max_iter': 100, 'pretrain_lr__multi_class': 'auto', 'pretrain_lr__n_jobs': None, 'pretrain_lr__penalty': 'l2', 'pretrain_lr__random_state': None, 'pretrain_lr__solver': 'lbfgs', 'pretrain_lr__target': 'creditability', 'pretrain_lr__tol': 0.0001, 'pretrain_lr__verbose': 0, 'pretrain_lr__warm_start': False, 'pretrain_lr': ITLubberLogisticRegression(target='creditability'), 'rate': 2, 'target': 'creditability', 'transer': &lt;toad.transform.WOETransformer object at 0x000002C34D407B90&gt;}</t>
         </is>
       </c>
     </row>
@@ -16864,197 +16864,197 @@
     <row r="68">
       <c r="B68" s="7" t="inlineStr">
         <is>
-          <t>credit_history</t>
+          <t>purpose</t>
         </is>
       </c>
       <c r="C68" s="7" t="n">
-        <v>0.7457</v>
+        <v>0.906</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>0.2025</v>
+        <v>0.2183</v>
       </c>
       <c r="E68" s="7" t="n">
-        <v>3.6834</v>
+        <v>4.1511</v>
       </c>
       <c r="F68" s="7" t="n">
-        <v>0.0002</v>
+        <v>0</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>0.3489</v>
+        <v>0.4782</v>
       </c>
       <c r="H68" s="7" t="n">
-        <v>1.1425</v>
+        <v>1.3338</v>
       </c>
       <c r="I68" s="7" t="n">
-        <v>1.078</v>
+        <v>1.0387</v>
       </c>
     </row>
     <row r="69">
       <c r="B69" s="9" t="inlineStr">
         <is>
-          <t>status_of_existing_checking_account</t>
+          <t>savings_account_and_bonds</t>
         </is>
       </c>
       <c r="C69" s="9" t="n">
-        <v>0.8066</v>
+        <v>0.6814</v>
       </c>
       <c r="D69" s="9" t="n">
-        <v>0.1281</v>
+        <v>0.2639</v>
       </c>
       <c r="E69" s="9" t="n">
-        <v>6.2976</v>
+        <v>2.5824</v>
       </c>
       <c r="F69" s="9" t="n">
-        <v>0</v>
+        <v>0.0098</v>
       </c>
       <c r="G69" s="9" t="n">
-        <v>0.5556</v>
+        <v>0.1642</v>
       </c>
       <c r="H69" s="9" t="n">
-        <v>1.0576</v>
+        <v>1.1986</v>
       </c>
       <c r="I69" s="9" t="n">
-        <v>1.1074</v>
+        <v>1.0595</v>
       </c>
     </row>
     <row r="70">
       <c r="B70" s="7" t="inlineStr">
         <is>
-          <t>housing</t>
+          <t>credit_history</t>
         </is>
       </c>
       <c r="C70" s="7" t="n">
-        <v>0.6862</v>
+        <v>0.7457</v>
       </c>
       <c r="D70" s="7" t="n">
-        <v>0.2889</v>
+        <v>0.2025</v>
       </c>
       <c r="E70" s="7" t="n">
-        <v>2.3755</v>
+        <v>3.6834</v>
       </c>
       <c r="F70" s="7" t="n">
-        <v>0.0175</v>
+        <v>0.0002</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>0.12</v>
+        <v>0.3489</v>
       </c>
       <c r="H70" s="7" t="n">
-        <v>1.2523</v>
+        <v>1.1425</v>
       </c>
       <c r="I70" s="7" t="n">
-        <v>1.0435</v>
+        <v>1.078</v>
       </c>
     </row>
     <row r="71">
       <c r="B71" s="9" t="inlineStr">
         <is>
-          <t>purpose</t>
+          <t>property</t>
         </is>
       </c>
       <c r="C71" s="9" t="n">
-        <v>0.906</v>
+        <v>0.7066</v>
       </c>
       <c r="D71" s="9" t="n">
-        <v>0.2183</v>
+        <v>0.3083</v>
       </c>
       <c r="E71" s="9" t="n">
-        <v>4.1511</v>
+        <v>2.2923</v>
       </c>
       <c r="F71" s="9" t="n">
-        <v>0</v>
+        <v>0.0219</v>
       </c>
       <c r="G71" s="9" t="n">
-        <v>0.4782</v>
+        <v>0.1024</v>
       </c>
       <c r="H71" s="9" t="n">
-        <v>1.3338</v>
+        <v>1.3108</v>
       </c>
       <c r="I71" s="9" t="n">
-        <v>1.0387</v>
+        <v>1.034</v>
       </c>
     </row>
     <row r="72">
       <c r="B72" s="7" t="inlineStr">
         <is>
-          <t>property</t>
+          <t>status_of_existing_checking_account</t>
         </is>
       </c>
       <c r="C72" s="7" t="n">
-        <v>0.7066</v>
+        <v>0.8066</v>
       </c>
       <c r="D72" s="7" t="n">
-        <v>0.3083</v>
+        <v>0.1281</v>
       </c>
       <c r="E72" s="7" t="n">
-        <v>2.2923</v>
+        <v>6.2976</v>
       </c>
       <c r="F72" s="7" t="n">
-        <v>0.0219</v>
+        <v>0</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>0.1024</v>
+        <v>0.5556</v>
       </c>
       <c r="H72" s="7" t="n">
-        <v>1.3108</v>
+        <v>1.0576</v>
       </c>
       <c r="I72" s="7" t="n">
-        <v>1.034</v>
+        <v>1.1074</v>
       </c>
     </row>
     <row r="73">
       <c r="B73" s="9" t="inlineStr">
         <is>
-          <t>savings_account_and_bonds</t>
+          <t>age_in_years</t>
         </is>
       </c>
       <c r="C73" s="9" t="n">
-        <v>0.6814</v>
+        <v>0.8222</v>
       </c>
       <c r="D73" s="9" t="n">
-        <v>0.2639</v>
+        <v>0.2942</v>
       </c>
       <c r="E73" s="9" t="n">
-        <v>2.5824</v>
+        <v>2.7946</v>
       </c>
       <c r="F73" s="9" t="n">
-        <v>0.0098</v>
+        <v>0.0052</v>
       </c>
       <c r="G73" s="9" t="n">
-        <v>0.1642</v>
+        <v>0.2455</v>
       </c>
       <c r="H73" s="9" t="n">
-        <v>1.1986</v>
+        <v>1.3989</v>
       </c>
       <c r="I73" s="9" t="n">
-        <v>1.0595</v>
+        <v>1.0713</v>
       </c>
     </row>
     <row r="74">
       <c r="B74" s="11" t="inlineStr">
         <is>
-          <t>age_in_years</t>
+          <t>housing</t>
         </is>
       </c>
       <c r="C74" s="11" t="n">
-        <v>0.8222</v>
+        <v>0.6862</v>
       </c>
       <c r="D74" s="11" t="n">
-        <v>0.2942</v>
+        <v>0.2889</v>
       </c>
       <c r="E74" s="11" t="n">
-        <v>2.7946</v>
+        <v>2.3755</v>
       </c>
       <c r="F74" s="11" t="n">
-        <v>0.0052</v>
+        <v>0.0175</v>
       </c>
       <c r="G74" s="11" t="n">
-        <v>0.2455</v>
+        <v>0.12</v>
       </c>
       <c r="H74" s="11" t="n">
-        <v>1.3989</v>
+        <v>1.2523</v>
       </c>
       <c r="I74" s="11" t="n">
-        <v>1.0713</v>
+        <v>1.0435</v>
       </c>
     </row>
     <row r="77">
@@ -17263,301 +17263,301 @@
     <row r="94">
       <c r="B94" s="26" t="inlineStr">
         <is>
-          <t>credit_history</t>
+          <t>purpose</t>
         </is>
       </c>
       <c r="C94" s="9" t="inlineStr">
         <is>
-          <t>信用历史</t>
+          <t>贷款目的</t>
         </is>
       </c>
       <c r="D94" s="26" t="inlineStr">
         <is>
-          <t>critical account/ other credits existing (not at this bank)</t>
+          <t>radio/television,furniture/equipment,car (used),repairs,retraining</t>
         </is>
       </c>
       <c r="E94" s="26" t="n">
-        <v>120.5116</v>
+        <v>95.1703</v>
       </c>
     </row>
     <row r="95">
       <c r="B95" s="25" t="inlineStr">
         <is>
-          <t>credit_history</t>
+          <t>purpose</t>
         </is>
       </c>
       <c r="C95" s="7" t="inlineStr">
         <is>
-          <t>信用历史</t>
+          <t>贷款目的</t>
         </is>
       </c>
       <c r="D95" s="25" t="inlineStr">
         <is>
-          <t>delay in paying off in the past,no credits taken/ all credits paid back duly,existing credits paid back duly till now,all credits at this bank paid back duly</t>
+          <t>domestic appliances,education,business,others,car (new)</t>
         </is>
       </c>
       <c r="E95" s="25" t="n">
-        <v>45.9673</v>
+        <v>26.5729</v>
       </c>
     </row>
     <row r="96">
       <c r="B96" s="26" t="inlineStr">
         <is>
-          <t>status_of_existing_checking_account</t>
+          <t>savings_account_and_bonds</t>
         </is>
       </c>
       <c r="C96" s="9" t="inlineStr">
         <is>
-          <t>支票账户状态</t>
+          <t>储蓄账户</t>
         </is>
       </c>
       <c r="D96" s="26" t="inlineStr">
         <is>
-          <t>no checking account,... &gt;= 200 DM / salary assignments for at least 1 year</t>
+          <t>500 &lt;= ... &lt; 1000 DM,... &gt;= 1000 DM,unknown/ no savings account</t>
         </is>
       </c>
       <c r="E96" s="26" t="n">
-        <v>132.8268</v>
+        <v>101.6595</v>
       </c>
     </row>
     <row r="97">
       <c r="B97" s="25" t="inlineStr">
         <is>
-          <t>status_of_existing_checking_account</t>
+          <t>savings_account_and_bonds</t>
         </is>
       </c>
       <c r="C97" s="7" t="inlineStr">
         <is>
-          <t>支票账户状态</t>
+          <t>储蓄账户</t>
         </is>
       </c>
       <c r="D97" s="25" t="inlineStr">
         <is>
-          <t>0 &lt;= ... &lt; 200 DM</t>
+          <t>... &lt; 100 DM,100 &lt;= ... &lt; 500 DM</t>
         </is>
       </c>
       <c r="E97" s="25" t="n">
-        <v>37.3467</v>
+        <v>51.2556</v>
       </c>
     </row>
     <row r="98">
       <c r="B98" s="26" t="inlineStr">
         <is>
-          <t>status_of_existing_checking_account</t>
+          <t>credit_history</t>
         </is>
       </c>
       <c r="C98" s="9" t="inlineStr">
         <is>
-          <t>支票账户状态</t>
+          <t>信用历史</t>
         </is>
       </c>
       <c r="D98" s="26" t="inlineStr">
         <is>
-          <t>... &lt; 0 DM</t>
+          <t>critical account/ other credits existing (not at this bank)</t>
         </is>
       </c>
       <c r="E98" s="26" t="n">
-        <v>9.431699999999999</v>
+        <v>120.5116</v>
       </c>
     </row>
     <row r="99">
       <c r="B99" s="25" t="inlineStr">
         <is>
-          <t>housing</t>
+          <t>credit_history</t>
         </is>
       </c>
       <c r="C99" s="7" t="inlineStr">
         <is>
-          <t>住房情况</t>
+          <t>信用历史</t>
         </is>
       </c>
       <c r="D99" s="25" t="inlineStr">
         <is>
-          <t>own</t>
+          <t>no credits taken/ all credits paid back duly,delay in paying off in the past,all credits at this bank paid back duly,existing credits paid back duly till now</t>
         </is>
       </c>
       <c r="E99" s="25" t="n">
-        <v>77.4657</v>
+        <v>45.9673</v>
       </c>
     </row>
     <row r="100">
       <c r="B100" s="26" t="inlineStr">
         <is>
-          <t>housing</t>
+          <t>property</t>
         </is>
       </c>
       <c r="C100" s="9" t="inlineStr">
         <is>
-          <t>住房情况</t>
+          <t>财产情况</t>
         </is>
       </c>
       <c r="D100" s="26" t="inlineStr">
         <is>
-          <t>for free,rent</t>
+          <t>real estate</t>
         </is>
       </c>
       <c r="E100" s="26" t="n">
-        <v>35.6204</v>
+        <v>97.8419</v>
       </c>
     </row>
     <row r="101">
       <c r="B101" s="25" t="inlineStr">
         <is>
-          <t>purpose</t>
+          <t>property</t>
         </is>
       </c>
       <c r="C101" s="7" t="inlineStr">
         <is>
-          <t>贷款目的</t>
+          <t>财产情况</t>
         </is>
       </c>
       <c r="D101" s="25" t="inlineStr">
         <is>
-          <t>furniture/equipment,radio/television,retraining,repairs,car (used)</t>
+          <t>building society savings agreement/ life insurance,car or other, not in attribute Savings account/bonds,unknown / no property</t>
         </is>
       </c>
       <c r="E101" s="25" t="n">
-        <v>95.1703</v>
+        <v>53.3921</v>
       </c>
     </row>
     <row r="102">
       <c r="B102" s="26" t="inlineStr">
         <is>
-          <t>purpose</t>
+          <t>status_of_existing_checking_account</t>
         </is>
       </c>
       <c r="C102" s="9" t="inlineStr">
         <is>
-          <t>贷款目的</t>
+          <t>支票账户状态</t>
         </is>
       </c>
       <c r="D102" s="26" t="inlineStr">
         <is>
-          <t>domestic appliances,others,car (new),education,business</t>
+          <t>no checking account,... &gt;= 200 DM / salary assignments for at least 1 year</t>
         </is>
       </c>
       <c r="E102" s="26" t="n">
-        <v>26.5729</v>
+        <v>132.8268</v>
       </c>
     </row>
     <row r="103">
       <c r="B103" s="25" t="inlineStr">
         <is>
-          <t>property</t>
+          <t>status_of_existing_checking_account</t>
         </is>
       </c>
       <c r="C103" s="7" t="inlineStr">
         <is>
-          <t>财产情况</t>
+          <t>支票账户状态</t>
         </is>
       </c>
       <c r="D103" s="25" t="inlineStr">
         <is>
-          <t>real estate</t>
+          <t>0 &lt;= ... &lt; 200 DM</t>
         </is>
       </c>
       <c r="E103" s="25" t="n">
-        <v>97.8419</v>
+        <v>37.3467</v>
       </c>
     </row>
     <row r="104">
       <c r="B104" s="26" t="inlineStr">
         <is>
-          <t>property</t>
+          <t>status_of_existing_checking_account</t>
         </is>
       </c>
       <c r="C104" s="9" t="inlineStr">
         <is>
-          <t>财产情况</t>
+          <t>支票账户状态</t>
         </is>
       </c>
       <c r="D104" s="26" t="inlineStr">
         <is>
-          <t>car or other, not in attribute Savings account/bonds,building society savings agreement/ life insurance,unknown / no property</t>
+          <t>... &lt; 0 DM</t>
         </is>
       </c>
       <c r="E104" s="26" t="n">
-        <v>53.3921</v>
+        <v>9.431699999999999</v>
       </c>
     </row>
     <row r="105">
       <c r="B105" s="25" t="inlineStr">
         <is>
-          <t>savings_account_and_bonds</t>
+          <t>age_in_years</t>
         </is>
       </c>
       <c r="C105" s="7" t="inlineStr">
         <is>
-          <t>储蓄账户</t>
+          <t>年龄</t>
         </is>
       </c>
       <c r="D105" s="25" t="inlineStr">
         <is>
-          <t>500 &lt;= ... &lt; 1000 DM,unknown/ no savings account,... &gt;= 1000 DM</t>
+          <t>[负无穷 , 35)</t>
         </is>
       </c>
       <c r="E105" s="25" t="n">
-        <v>101.6595</v>
+        <v>44.6394</v>
       </c>
     </row>
     <row r="106">
       <c r="B106" s="26" t="inlineStr">
         <is>
-          <t>savings_account_and_bonds</t>
+          <t>age_in_years</t>
         </is>
       </c>
       <c r="C106" s="9" t="inlineStr">
         <is>
-          <t>储蓄账户</t>
+          <t>年龄</t>
         </is>
       </c>
       <c r="D106" s="26" t="inlineStr">
         <is>
-          <t>100 &lt;= ... &lt; 500 DM,... &lt; 100 DM</t>
+          <t>[35 , 正无穷)</t>
         </is>
       </c>
       <c r="E106" s="26" t="n">
-        <v>51.2556</v>
+        <v>92.5921</v>
       </c>
     </row>
     <row r="107">
       <c r="B107" s="25" t="inlineStr">
         <is>
-          <t>age_in_years</t>
+          <t>housing</t>
         </is>
       </c>
       <c r="C107" s="7" t="inlineStr">
         <is>
-          <t>年龄</t>
+          <t>住房情况</t>
         </is>
       </c>
       <c r="D107" s="25" t="inlineStr">
         <is>
-          <t>[负无穷 , 35)</t>
+          <t>own</t>
         </is>
       </c>
       <c r="E107" s="25" t="n">
-        <v>44.6394</v>
+        <v>77.4657</v>
       </c>
     </row>
     <row r="108">
       <c r="B108" s="30" t="inlineStr">
         <is>
-          <t>age_in_years</t>
+          <t>housing</t>
         </is>
       </c>
       <c r="C108" s="18" t="inlineStr">
         <is>
-          <t>年龄</t>
+          <t>住房情况</t>
         </is>
       </c>
       <c r="D108" s="30" t="inlineStr">
         <is>
-          <t>[35 , 正无穷)</t>
+          <t>rent,for free</t>
         </is>
       </c>
       <c r="E108" s="30" t="n">
-        <v>92.5921</v>
+        <v>35.6204</v>
       </c>
     </row>
   </sheetData>

</xml_diff>